<commit_message>
Atualização automática leitura Parcial_Piracicaba.xlsx
</commit_message>
<xml_diff>
--- a/dashboard/leitura/Parcial_Piracicaba.xlsx
+++ b/dashboard/leitura/Parcial_Piracicaba.xlsx
@@ -608,77 +608,77 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MARCELO DO PRADO CAMARGO</t>
+          <t>ALEX JONYRIGO</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>198</v>
+        <v>318</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>175</v>
+        <v>301</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>88.38</v>
+        <v>94.65000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ALEX JONYRIGO</t>
+          <t>HENRIQUE DOS SANTOS DIAS</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>318</v>
+        <v>496</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>301</v>
+        <v>478</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>94.65000000000001</v>
+        <v>96.37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HENRIQUE DOS SANTOS DIAS</t>
+          <t>ADAO RIBEIRO</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>496</v>
+        <v>80</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>478</v>
+        <v>78</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>96.37</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ADAO RIBEIRO</t>
+          <t>MARCELO DO PRADO CAMARGO</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>80</v>
+        <v>198</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>78</v>
+        <v>195</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>97.5</v>
+        <v>98.48</v>
       </c>
     </row>
     <row r="11">

</xml_diff>